<commit_message>
fix(contenu): précise les concerts publics, harmonise les dates et corrige les textes et la setlist
</commit_message>
<xml_diff>
--- a/src/content/setListNevro.xlsx
+++ b/src/content/setListNevro.xlsx
@@ -59,37 +59,37 @@
     <t>Névrosyne</t>
   </si>
   <si>
-    <t>7 nation army</t>
-  </si>
-  <si>
-    <t>White stripes</t>
-  </si>
-  <si>
-    <t>A l’ombre</t>
+    <t>Seven Nation Army</t>
+  </si>
+  <si>
+    <t>The White Stripes</t>
+  </si>
+  <si>
+    <t>À l’ombre</t>
   </si>
   <si>
     <t>Mademoiselle K</t>
   </si>
   <si>
-    <t>A little less conversation</t>
+    <t>A Little Less Conversation</t>
   </si>
   <si>
     <t>Elvis Presley</t>
   </si>
   <si>
-    <t>Are U gonna be my girl</t>
+    <t>Are You Gonna Be My Girl</t>
   </si>
   <si>
     <t>Jet</t>
   </si>
   <si>
-    <t>Are U gonna go my way</t>
+    <t>Are You Gonna Go My Way</t>
   </si>
   <si>
     <t>Lenny Kravitz</t>
   </si>
   <si>
-    <t>Back to black</t>
+    <t>Back to Black</t>
   </si>
   <si>
     <t>Amy Winehouse</t>
@@ -101,19 +101,19 @@
     <t>Billie Eilish</t>
   </si>
   <si>
-    <t>Beggin'</t>
-  </si>
-  <si>
-    <t>Maneskin</t>
-  </si>
-  <si>
-    <t>Big white gate</t>
+    <t>Beggin’</t>
+  </si>
+  <si>
+    <t>Måneskin</t>
+  </si>
+  <si>
+    <t>Big White Gate</t>
   </si>
   <si>
     <t>Grace Potter</t>
   </si>
   <si>
-    <t>Boyz don't cry</t>
+    <t>Boys Don’t Cry</t>
   </si>
   <si>
     <t>The Cure</t>
@@ -125,7 +125,7 @@
     <t>Nirvana</t>
   </si>
   <si>
-    <t>Ca c’est vraiment toi</t>
+    <t>Ça (c’est vraiment toi)</t>
   </si>
   <si>
     <t>Colors</t>
@@ -134,25 +134,25 @@
     <t>Black Pumas</t>
   </si>
   <si>
-    <t>Come out and play</t>
-  </si>
-  <si>
-    <t>Offspring</t>
-  </si>
-  <si>
-    <t>Mathieu Chédid</t>
-  </si>
-  <si>
-    <t>Dancing barefoot</t>
+    <t>Come Out and Play</t>
+  </si>
+  <si>
+    <t>The Offspring</t>
+  </si>
+  <si>
+    <t>-M- (Matthieu Chedid)</t>
+  </si>
+  <si>
+    <t>Dancing Barefoot</t>
   </si>
   <si>
     <t>Patti Smith</t>
   </si>
   <si>
-    <t>Girls just want to have fun</t>
-  </si>
-  <si>
-    <t>Cyndi Lauper Nevro ver</t>
+    <t>Girls Just Want to Have Fun</t>
+  </si>
+  <si>
+    <t>Cyndi Lauper – version Névrosyne</t>
   </si>
   <si>
     <t>Goldfish</t>
@@ -161,28 +161,28 @@
     <t>Heartbreaker</t>
   </si>
   <si>
-    <t>Pat Bénatar</t>
-  </si>
-  <si>
-    <t>Here comes the rain again</t>
+    <t>Pat Benatar</t>
+  </si>
+  <si>
+    <t>Here Comes the Rain Again</t>
   </si>
   <si>
     <t>Eurythmics</t>
   </si>
   <si>
-    <t>I'm Picky</t>
+    <t>I’m Picky</t>
   </si>
   <si>
     <t>Shaka Ponk</t>
   </si>
   <si>
-    <t>I'm shipping up to boston</t>
+    <t>I’m Shipping Up to Boston</t>
   </si>
   <si>
     <t>Dropkick Murphys</t>
   </si>
   <si>
-    <t>In my place</t>
+    <t>In My Place</t>
   </si>
   <si>
     <t>Coldplay</t>
@@ -191,10 +191,10 @@
     <t>J’t’emmène au vent</t>
   </si>
   <si>
-    <t>Louise Attaque – Nevro ver.</t>
-  </si>
-  <si>
-    <t>Je dis M</t>
+    <t>Louise Attaque – version Névrosyne</t>
+  </si>
+  <si>
+    <t>Je dis aime</t>
   </si>
   <si>
     <t>Kids in America</t>
@@ -203,46 +203,46 @@
     <t>Kim Wilde</t>
   </si>
   <si>
-    <t>Killing in the name</t>
+    <t>Killing in the Name</t>
   </si>
   <si>
     <t>Rage Against the Machine</t>
   </si>
   <si>
-    <t>L'auvergnat + Bella Ciao</t>
-  </si>
-  <si>
-    <t>Brassens + ?</t>
-  </si>
-  <si>
-    <t>L'aventurier</t>
+    <t>L’Auvergnat + Bella Ciao</t>
+  </si>
+  <si>
+    <t>Georges Brassens + chant partisan italien</t>
+  </si>
+  <si>
+    <t>L’Aventurier</t>
   </si>
   <si>
     <t>Indochine</t>
   </si>
   <si>
-    <t>Make it wit chu</t>
-  </si>
-  <si>
-    <t>Queens of the stone age</t>
-  </si>
-  <si>
-    <t>Money for nothing</t>
+    <t>Make It Wit Chu</t>
+  </si>
+  <si>
+    <t>Queens of the Stone Age</t>
+  </si>
+  <si>
+    <t>Money for Nothing</t>
   </si>
   <si>
     <t>Dire Straits</t>
   </si>
   <si>
-    <t>Never look back</t>
+    <t>Never Look Back</t>
   </si>
   <si>
     <t>Personal Jesus</t>
   </si>
   <si>
-    <t>Ko ko mo ver.</t>
-  </si>
-  <si>
-    <t>Plug in baby</t>
+    <t>Depeche Mode – version Ko Ko Mo</t>
+  </si>
+  <si>
+    <t>Plug In Baby</t>
   </si>
   <si>
     <t>Muse</t>
@@ -251,19 +251,19 @@
     <t>Psycho</t>
   </si>
   <si>
-    <t>Shadow without you</t>
+    <t>Shadow Without You</t>
   </si>
   <si>
     <t>Linkin Park &amp; U2</t>
   </si>
   <si>
-    <t>six blade knife</t>
-  </si>
-  <si>
-    <t>Dire straits</t>
-  </si>
-  <si>
-    <t>Smells like teen spirits</t>
+    <t>Six Blade Knife</t>
+  </si>
+  <si>
+    <t>Dire Straits</t>
+  </si>
+  <si>
+    <t>Smells Like Teen Spirit</t>
   </si>
   <si>
     <t>Song 2</t>
@@ -281,16 +281,16 @@
     <t>Sweet Dreams</t>
   </si>
   <si>
-    <t>Eurythmics &amp; Marylin Manson</t>
+    <t>Eurythmics &amp; Marilyn Manson</t>
   </si>
   <si>
     <t>Tainted Love</t>
   </si>
   <si>
-    <t>Soft Cell - Nevro ver</t>
-  </si>
-  <si>
-    <t>Take me out</t>
+    <t>Soft Cell – version Névrosyne</t>
+  </si>
+  <si>
+    <t>Take Me Out</t>
   </si>
   <si>
     <t>Franz Ferdinand</t>
@@ -302,25 +302,25 @@
     <t>Jean-Louis Aubert</t>
   </si>
   <si>
-    <t>Time is running out</t>
+    <t>Time Is Running Out</t>
   </si>
   <si>
     <t>Toxicity</t>
   </si>
   <si>
-    <t>System of a down</t>
-  </si>
-  <si>
-    <t>Walk like an Egyptian</t>
-  </si>
-  <si>
-    <t>Bangles</t>
-  </si>
-  <si>
-    <t>War Paranoid</t>
-  </si>
-  <si>
-    <t>Black Sabath</t>
+    <t>System of a Down</t>
+  </si>
+  <si>
+    <t>Walk Like an Egyptian</t>
+  </si>
+  <si>
+    <t>The Bangles</t>
+  </si>
+  <si>
+    <t>War Pigs / Paranoid</t>
+  </si>
+  <si>
+    <t>Black Sabbath</t>
   </si>
   <si>
     <t>Waterfalls</t>
@@ -338,52 +338,52 @@
     <t>Shout</t>
   </si>
   <si>
-    <t>Tears for fear - Nevro ver</t>
-  </si>
-  <si>
-    <t>Téléphone  - Nevro ver</t>
-  </si>
-  <si>
-    <t>Despair Hangover and Ecstasy</t>
-  </si>
-  <si>
-    <t>The Do - Nevro ver</t>
+    <t>Tears for Fears – version Névrosyne</t>
+  </si>
+  <si>
+    <t>Téléphone – version Névrosyne</t>
+  </si>
+  <si>
+    <t>Despair, Hangover &amp; Ecstasy</t>
+  </si>
+  <si>
+    <t>The Dø – version Névrosyne</t>
   </si>
   <si>
     <t>Get Free</t>
   </si>
   <si>
-    <t>The vines</t>
-  </si>
-  <si>
-    <t>Girls and Boys</t>
-  </si>
-  <si>
-    <t>Blur - Nevro ver</t>
-  </si>
-  <si>
-    <t>La isla Bonita</t>
-  </si>
-  <si>
-    <t>Madonna - Nevro ver</t>
+    <t>The Vines</t>
+  </si>
+  <si>
+    <t>Girls &amp; Boys</t>
+  </si>
+  <si>
+    <t>Blur – version Névrosyne</t>
+  </si>
+  <si>
+    <t>La Isla Bonita</t>
+  </si>
+  <si>
+    <t>Madonna – version Névrosyne</t>
   </si>
   <si>
     <t>Smalltown Forest</t>
   </si>
   <si>
-    <t>The Cure / Jimmy summerville - Nevro ver</t>
-  </si>
-  <si>
-    <t>Whole lotta Rosie</t>
-  </si>
-  <si>
-    <t>ACDC</t>
-  </si>
-  <si>
-    <t>Wonderfull life</t>
-  </si>
-  <si>
-    <t>Black - Nevro ver</t>
+    <t>The Cure / Jimmy Somerville – version Névrosyne</t>
+  </si>
+  <si>
+    <t>Whole Lotta Rosie</t>
+  </si>
+  <si>
+    <t>AC/DC</t>
+  </si>
+  <si>
+    <t>Wonderful Life</t>
+  </si>
+  <si>
+    <t>Black – version Névrosyne</t>
   </si>
 </sst>
 </file>

</xml_diff>